<commit_message>
fix: 修正CPU3版本显示与液位参数单位（CPU2 V0.17.2.0 / CPU3 V0.18.2.0）
版本：
- CPU2：V0.17.2.0（历史提交编号）
- CPU3：V0.18.2.0（历史提交编号）

协议版本/兼容性：
- 涉及外部 Modbus、DSM 或瓦锡兰通信；接口口径以该历史提交的代码树为准。

本次修改：
- 更新 CPU3 版本标识和显示字库。
- 修正液位模式、修正参数单位及姿态角显示条件。

验证：
- 提交差异复核：通过；本次仅重写说明，代码树保持不变。
</commit_message>
<xml_diff>
--- a/LTD_DISPLAY_CPU3/readme/LTD故障代码表.xlsx
+++ b/LTD_DISPLAY_CPU3/readme/LTD故障代码表.xlsx
@@ -4070,6 +4070,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -13511,8 +13514,8 @@
       <c r="K74" t="s">
         <v>450</v>
       </c>
-      <c r="L74" t="s">
-        <v>436</v>
+      <c r="L74" s="19" t="s">
+        <v>553</v>
       </c>
       <c r="M74" t="s">
         <v>442</v>
@@ -13561,8 +13564,8 @@
       <c r="K75" t="s">
         <v>450</v>
       </c>
-      <c r="L75" t="s">
-        <v>436</v>
+      <c r="L75" s="19" t="s">
+        <v>560</v>
       </c>
       <c r="M75" t="s">
         <v>442</v>
@@ -14409,7 +14412,7 @@
         <v>516</v>
       </c>
       <c r="K94" t="s">
-        <v>450</v>
+        <v>436</v>
       </c>
       <c r="L94" t="s">
         <v>436</v>
@@ -14459,7 +14462,7 @@
         <v>516</v>
       </c>
       <c r="K95" t="s">
-        <v>450</v>
+        <v>436</v>
       </c>
       <c r="L95" t="s">
         <v>436</v>
@@ -14509,7 +14512,7 @@
         <v>516</v>
       </c>
       <c r="K96" t="s">
-        <v>450</v>
+        <v>436</v>
       </c>
       <c r="L96" t="s">
         <v>436</v>
@@ -14559,7 +14562,7 @@
         <v>516</v>
       </c>
       <c r="K97" t="s">
-        <v>450</v>
+        <v>436</v>
       </c>
       <c r="L97" t="s">
         <v>436</v>

</xml_diff>

<commit_message>
feat: 增加水位快速寻找与跟随方式（CPU2 V0.19.0.0 / CPU3 V0.20.0.0）
版本：
- CPU2：V0.19.0.0（历史提交编号）
- CPU3：V0.20.0.0（历史提交编号）

协议版本/兼容性：
- 涉及 DSM、LTD 或无线传感器通信；协议口径以该历史提交的代码树为准。

本次修改：
- 新增水位快速寻找、状态翻转判定和跟随流程。
- 同步 CPU2/CPU3 水位模式、稳定阈值及罐底参数。

验证：
- 提交差异复核：通过；本次仅重写说明，代码树保持不变。
</commit_message>
<xml_diff>
--- a/LTD_DISPLAY_CPU3/readme/LTD故障代码表.xlsx
+++ b/LTD_DISPLAY_CPU3/readme/LTD故障代码表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255" activeTab="4"/>
+    <workbookView windowWidth="28800" windowHeight="12255" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="总表" sheetId="1" r:id="rId1"/>
@@ -2505,13 +2505,13 @@
     <t>(uint8_t*)"WaterTankH"},</t>
   </si>
   <si>
-    <t>{(uint8_t*)"水位探头距差",</t>
-  </si>
-  <si>
-    <t>COM_NUM_DEVICEPARAM_WATER_LEVEL_SENSOR_DISTANCE_DIFF,</t>
-  </si>
-  <si>
-    <t>HOLDREGISTER_DEVICEPARAM_WATER_LEVEL_SENSOR_DISTANCE_DIFF,</t>
+    <t>{(uint8_t*)"水位测量方式",</t>
+  </si>
+  <si>
+    <t>COM_NUM_DEVICEPARAM_WATER_LEVEL_MODE,</t>
+  </si>
+  <si>
+    <t>HOLDREGISTER_DEVICEPARAM_WATER_LEVEL_MODE,</t>
   </si>
   <si>
     <t>(uint8_t*)"WaterSenDiff"},</t>
@@ -2553,13 +2553,13 @@
     <t>(uint8_t*)"ZeroCap"},</t>
   </si>
   <si>
-    <t>{(uint8_t*)"保留15",</t>
-  </si>
-  <si>
-    <t>COM_NUM_DEVICEPARAM_RESERVED15,</t>
-  </si>
-  <si>
-    <t>HOLDREGISTER_DEVICEPARAM_RESERVED15,</t>
+    <t>{(uint8_t*)"水位稳定阈值",</t>
+  </si>
+  <si>
+    <t>COM_NUM_DEVICEPARAM_WATER_STABLE_THRESHOLD,</t>
+  </si>
+  <si>
+    <t>HOLDREGISTER_DEVICEPARAM_WATER_STABLE_THRESHOLD,</t>
   </si>
   <si>
     <t>(uint8_t*)"Rsv15"},</t>
@@ -12703,28 +12703,28 @@
         <v>440</v>
       </c>
       <c r="H56" t="s">
-        <v>803</v>
+        <v>436</v>
       </c>
       <c r="I56" t="s">
-        <v>804</v>
+        <v>436</v>
       </c>
       <c r="J56" t="s">
-        <v>516</v>
+        <v>441</v>
       </c>
       <c r="K56" t="s">
+        <v>436</v>
+      </c>
+      <c r="L56" t="s">
+        <v>436</v>
+      </c>
+      <c r="M56" t="s">
+        <v>442</v>
+      </c>
+      <c r="N56" t="s">
+        <v>443</v>
+      </c>
+      <c r="O56" t="s">
         <v>450</v>
-      </c>
-      <c r="L56" t="s">
-        <v>436</v>
-      </c>
-      <c r="M56" t="s">
-        <v>442</v>
-      </c>
-      <c r="N56" t="s">
-        <v>443</v>
-      </c>
-      <c r="O56" t="s">
-        <v>451</v>
       </c>
       <c r="P56" t="s">
         <v>441</v>
@@ -12968,7 +12968,7 @@
         <v>436</v>
       </c>
       <c r="M61" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="N61" t="s">
         <v>443</v>
@@ -13009,22 +13009,22 @@
         <v>436</v>
       </c>
       <c r="J62" t="s">
-        <v>441</v>
+        <v>516</v>
       </c>
       <c r="K62" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
       <c r="L62" t="s">
         <v>436</v>
       </c>
       <c r="M62" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="N62" t="s">
         <v>443</v>
       </c>
       <c r="O62" t="s">
-        <v>444</v>
+        <v>562</v>
       </c>
       <c r="P62" t="s">
         <v>441</v>

</xml_diff>